<commit_message>
refactor: ajustar planilha de horas extras para controle por semana (52 semanas + total)
</commit_message>
<xml_diff>
--- a/HORARIO/HORAS_EXTRAS_2026.xlsx
+++ b/HORARIO/HORAS_EXTRAS_2026.xlsx
@@ -16,10 +16,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
-  </numFmts>
-  <fonts count="5">
+  <numFmts count="0"/>
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -42,6 +40,10 @@
     <font>
       <name val="Calibri"/>
       <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -96,7 +98,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -105,15 +107,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -122,11 +121,11 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -494,11 +493,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -507,7 +506,7 @@
     <row r="1" ht="25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CONTROLE DE HORAS EXTRAS</t>
+          <t>CONTROLE DE HORAS EXTRAS POR SEMANA — 2026</t>
         </is>
       </c>
     </row>
@@ -515,17 +514,17 @@
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Mês</t>
+          <t>Semana</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
+          <t>Período (Seg–Dom)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
           <t>Horas Extras</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Data do Lançamento</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -542,160 +541,808 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Janeiro</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr"/>
+          <t>Semana 1</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>29/12 — 04/01/2026</t>
+        </is>
+      </c>
       <c r="C4" s="5" t="inlineStr"/>
-      <c r="D4" s="6" t="inlineStr"/>
-      <c r="E4" s="7" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>Fevereiro</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr"/>
+          <t>Semana 2</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>05/01 — 11/01/2026</t>
+        </is>
+      </c>
       <c r="C5" s="5" t="inlineStr"/>
-      <c r="D5" s="6" t="inlineStr"/>
-      <c r="E5" s="7" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Março</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr"/>
+          <t>Semana 3</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>12/01 — 18/01/2026</t>
+        </is>
+      </c>
       <c r="C6" s="5" t="inlineStr"/>
-      <c r="D6" s="6" t="inlineStr"/>
-      <c r="E6" s="7" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Abril</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr"/>
+          <t>Semana 4</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>19/01 — 25/01/2026</t>
+        </is>
+      </c>
       <c r="C7" s="5" t="inlineStr"/>
-      <c r="D7" s="6" t="inlineStr"/>
-      <c r="E7" s="7" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>Maio</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr"/>
+          <t>Semana 5</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>26/01 — 01/02/2026</t>
+        </is>
+      </c>
       <c r="C8" s="5" t="inlineStr"/>
-      <c r="D8" s="6" t="inlineStr"/>
-      <c r="E8" s="7" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Junho</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr"/>
+          <t>Semana 6</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>02/02 — 08/02/2026</t>
+        </is>
+      </c>
       <c r="C9" s="5" t="inlineStr"/>
-      <c r="D9" s="6" t="inlineStr"/>
-      <c r="E9" s="7" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Julho</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr"/>
+          <t>Semana 7</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>09/02 — 15/02/2026</t>
+        </is>
+      </c>
       <c r="C10" s="5" t="inlineStr"/>
-      <c r="D10" s="6" t="inlineStr"/>
-      <c r="E10" s="7" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>Agosto</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr"/>
+          <t>Semana 8</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>16/02 — 22/02/2026</t>
+        </is>
+      </c>
       <c r="C11" s="5" t="inlineStr"/>
-      <c r="D11" s="6" t="inlineStr"/>
-      <c r="E11" s="7" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Setembro</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr"/>
+          <t>Semana 9</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>23/02 — 01/03/2026</t>
+        </is>
+      </c>
       <c r="C12" s="5" t="inlineStr"/>
-      <c r="D12" s="6" t="inlineStr"/>
-      <c r="E12" s="7" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Outubro</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr"/>
+          <t>Semana 10</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>02/03 — 08/03/2026</t>
+        </is>
+      </c>
       <c r="C13" s="5" t="inlineStr"/>
-      <c r="D13" s="6" t="inlineStr"/>
-      <c r="E13" s="7" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Novembro</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr"/>
+          <t>Semana 11</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>09/03 — 15/03/2026</t>
+        </is>
+      </c>
       <c r="C14" s="5" t="inlineStr"/>
-      <c r="D14" s="6" t="inlineStr"/>
-      <c r="E14" s="7" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Dezembro</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr"/>
+          <t>Semana 12</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>16/03 — 22/03/2026</t>
+        </is>
+      </c>
       <c r="C15" s="5" t="inlineStr"/>
-      <c r="D15" s="6" t="inlineStr"/>
-      <c r="E15" s="7" t="inlineStr"/>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B16" s="9">
-        <f>SUM(B4:B15)</f>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Semana 13</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>23/03 — 29/03/2026</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Semana 14</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>30/03 — 05/04/2026</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Semana 15</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>06/04 — 12/04/2026</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Semana 16</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>13/04 — 19/04/2026</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Semana 17</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>20/04 — 26/04/2026</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Semana 18</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>27/04 — 03/05/2026</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Semana 19</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>04/05 — 10/05/2026</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr"/>
+      <c r="D22" s="3" t="inlineStr"/>
+      <c r="E22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Semana 20</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>11/05 — 17/05/2026</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr"/>
+      <c r="D23" s="3" t="inlineStr"/>
+      <c r="E23" s="6" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Semana 21</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>18/05 — 24/05/2026</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Semana 22</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>25/05 — 31/05/2026</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr"/>
+      <c r="E25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Semana 23</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>01/06 — 07/06/2026</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="6" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Semana 24</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>08/06 — 14/06/2026</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr"/>
+      <c r="E27" s="6" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Semana 25</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>15/06 — 21/06/2026</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr"/>
+      <c r="E28" s="6" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>Semana 26</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>22/06 — 28/06/2026</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr"/>
+      <c r="D29" s="3" t="inlineStr"/>
+      <c r="E29" s="6" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Semana 27</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>29/06 — 05/07/2026</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr"/>
+      <c r="D30" s="3" t="inlineStr"/>
+      <c r="E30" s="6" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>Semana 28</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>06/07 — 12/07/2026</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr"/>
+      <c r="D31" s="3" t="inlineStr"/>
+      <c r="E31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>Semana 29</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>13/07 — 19/07/2026</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr"/>
+      <c r="D32" s="3" t="inlineStr"/>
+      <c r="E32" s="6" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>Semana 30</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>20/07 — 26/07/2026</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr"/>
+      <c r="D33" s="3" t="inlineStr"/>
+      <c r="E33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>Semana 31</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>27/07 — 02/08/2026</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr"/>
+      <c r="D34" s="3" t="inlineStr"/>
+      <c r="E34" s="6" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>Semana 32</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>03/08 — 09/08/2026</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr"/>
+      <c r="D35" s="3" t="inlineStr"/>
+      <c r="E35" s="6" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>Semana 33</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>10/08 — 16/08/2026</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr"/>
+      <c r="D36" s="3" t="inlineStr"/>
+      <c r="E36" s="6" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Semana 34</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>17/08 — 23/08/2026</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr"/>
+      <c r="D37" s="3" t="inlineStr"/>
+      <c r="E37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>Semana 35</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>24/08 — 30/08/2026</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr"/>
+      <c r="D38" s="3" t="inlineStr"/>
+      <c r="E38" s="6" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Semana 36</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="inlineStr">
+        <is>
+          <t>31/08 — 06/09/2026</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr"/>
+      <c r="D39" s="3" t="inlineStr"/>
+      <c r="E39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Semana 37</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>07/09 — 13/09/2026</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr"/>
+      <c r="D40" s="3" t="inlineStr"/>
+      <c r="E40" s="6" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Semana 38</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>14/09 — 20/09/2026</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr"/>
+      <c r="D41" s="3" t="inlineStr"/>
+      <c r="E41" s="6" t="inlineStr"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Semana 39</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>21/09 — 27/09/2026</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr"/>
+      <c r="D42" s="3" t="inlineStr"/>
+      <c r="E42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>Semana 40</t>
+        </is>
+      </c>
+      <c r="B43" s="4" t="inlineStr">
+        <is>
+          <t>28/09 — 04/10/2026</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr"/>
+      <c r="D43" s="3" t="inlineStr"/>
+      <c r="E43" s="6" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Semana 41</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>05/10 — 11/10/2026</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr"/>
+      <c r="D44" s="3" t="inlineStr"/>
+      <c r="E44" s="6" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
+          <t>Semana 42</t>
+        </is>
+      </c>
+      <c r="B45" s="4" t="inlineStr">
+        <is>
+          <t>12/10 — 18/10/2026</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr"/>
+      <c r="D45" s="3" t="inlineStr"/>
+      <c r="E45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>Semana 43</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>19/10 — 25/10/2026</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr"/>
+      <c r="D46" s="3" t="inlineStr"/>
+      <c r="E46" s="6" t="inlineStr"/>
+    </row>
+    <row r="47" ht="20" customHeight="1">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>Semana 44</t>
+        </is>
+      </c>
+      <c r="B47" s="4" t="inlineStr">
+        <is>
+          <t>26/10 — 01/11/2026</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr"/>
+      <c r="D47" s="3" t="inlineStr"/>
+      <c r="E47" s="6" t="inlineStr"/>
+    </row>
+    <row r="48" ht="20" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>Semana 45</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>02/11 — 08/11/2026</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr"/>
+      <c r="D48" s="3" t="inlineStr"/>
+      <c r="E48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="3" t="inlineStr">
+        <is>
+          <t>Semana 46</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>09/11 — 15/11/2026</t>
+        </is>
+      </c>
+      <c r="C49" s="5" t="inlineStr"/>
+      <c r="D49" s="3" t="inlineStr"/>
+      <c r="E49" s="6" t="inlineStr"/>
+    </row>
+    <row r="50" ht="20" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>Semana 47</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>16/11 — 22/11/2026</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr"/>
+      <c r="D50" s="3" t="inlineStr"/>
+      <c r="E50" s="6" t="inlineStr"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="3" t="inlineStr">
+        <is>
+          <t>Semana 48</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>23/11 — 29/11/2026</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="inlineStr"/>
+      <c r="D51" s="3" t="inlineStr"/>
+      <c r="E51" s="6" t="inlineStr"/>
+    </row>
+    <row r="52" ht="20" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>Semana 49</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>30/11 — 06/12/2026</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr"/>
+      <c r="D52" s="3" t="inlineStr"/>
+      <c r="E52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53" ht="20" customHeight="1">
+      <c r="A53" s="3" t="inlineStr">
+        <is>
+          <t>Semana 50</t>
+        </is>
+      </c>
+      <c r="B53" s="4" t="inlineStr">
+        <is>
+          <t>07/12 — 13/12/2026</t>
+        </is>
+      </c>
+      <c r="C53" s="5" t="inlineStr"/>
+      <c r="D53" s="3" t="inlineStr"/>
+      <c r="E53" s="6" t="inlineStr"/>
+    </row>
+    <row r="54" ht="20" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>Semana 51</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>14/12 — 20/12/2026</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr"/>
+      <c r="D54" s="3" t="inlineStr"/>
+      <c r="E54" s="6" t="inlineStr"/>
+    </row>
+    <row r="55" ht="20" customHeight="1">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>Semana 52</t>
+        </is>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>21/12 — 27/12/2026</t>
+        </is>
+      </c>
+      <c r="C55" s="5" t="inlineStr"/>
+      <c r="D55" s="3" t="inlineStr"/>
+      <c r="E55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>TOTAL (52 semanas)</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n"/>
+      <c r="C56" s="9">
+        <f>SUM(C4:C55)</f>
         <v/>
       </c>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-    </row>
-    <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
-        <is>
-          <t>⚠️ Preench Hora Extras com decimais (ex: 2.5 = 2h30min) | Lançado: Digite 'Sim' ou 'Não' | Data: DD/MM/YYYY</t>
+      <c r="D56" s="8" t="n"/>
+      <c r="E56" s="8" t="n"/>
+    </row>
+    <row r="58" ht="30" customHeight="1">
+      <c r="A58" s="10" t="inlineStr">
+        <is>
+          <t>⚠️ Preencha Horas Extras com decimais (ex: 2.5 = 2h30min) | Lançado: Digite 'Sim' ou 'Não' | Período já calculado automaticamente</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A58:E58"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>